<commit_message>
fix(testdoku): Sicherheitskreise im Klemmenplan und Signalgraph, Klemmen aus dem Modell, Kanalnummern, --refresh raeumt alte Fehler ab
- Klemmenplan: je Sicherheitskreis Beginn/Ende beider Kanaele; Signalgraph wertet S12/S22 eines
  Sicherheitsrelais als Eingang (Not-Halt -> Relais -> E -> Freigabe -> Umrichter)
- Fehlertexte nennen Klemmen ueber {term:Adresse}, nicht mehr von Hand (PM1-AR nannte falsche Klemmen)
- DI/DO-Fortsetzungsblaetter zaehlen die Kanaele weiter; CPU -A1 als Symbol; Klemmenbeschriftung ueber dem Draht
- Lader: Maschine vor dem Upload pruefen, --refresh loescht importierte Fehler, 'failed' wird gemeldet

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/examples/aufrollung/02_Stueckliste_PM1-AR.xlsx
+++ b/examples/aufrollung/02_Stueckliste_PM1-AR.xlsx
@@ -1800,7 +1800,7 @@
       </c>
       <c r="F48" t="inlineStr">
         <is>
-          <t>/3.3</t>
+          <t>/7.1</t>
         </is>
       </c>
     </row>
@@ -1962,7 +1962,7 @@
       </c>
       <c r="B54" t="inlineStr">
         <is>
-          <t>Klemmleiste Feldgeraete (Sensoren, Taster, Ventile, Umrichter-Signale)</t>
+          <t>Klemmleiste Feldgeraete (Sensoren, Taster, Ventile, Umrichter-Signale, Sicherheitskreise)</t>
         </is>
       </c>
       <c r="C54" t="inlineStr">
@@ -1971,7 +1971,7 @@
         </is>
       </c>
       <c r="D54" t="n">
-        <v>34</v>
+        <v>42</v>
       </c>
       <c r="E54" t="inlineStr">
         <is>
@@ -1980,7 +1980,7 @@
       </c>
       <c r="F54" t="inlineStr">
         <is>
-          <t>/7.3</t>
+          <t>/5.2</t>
         </is>
       </c>
     </row>

</xml_diff>